<commit_message>
Sprint 217 performance results added
</commit_message>
<xml_diff>
--- a/PerformanceReports/GET_PERFORMANCE_API_REPORT.xlsx
+++ b/PerformanceReports/GET_PERFORMANCE_API_REPORT.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="835" uniqueCount="238">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="853" uniqueCount="246">
   <si>
     <t xml:space="preserve">Run Number</t>
   </si>
@@ -456,6 +456,15 @@
     <t xml:space="preserve">10:49:19</t>
   </si>
   <si>
+    <t xml:space="preserve">Sprint_217</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-04-22</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10:47:48</t>
+  </si>
+  <si>
     <t xml:space="preserve">11:53:AM</t>
   </si>
   <si>
@@ -513,6 +522,9 @@
     <t xml:space="preserve">10:50:56</t>
   </si>
   <si>
+    <t xml:space="preserve">11:10:38</t>
+  </si>
+  <si>
     <t xml:space="preserve">14:25:00</t>
   </si>
   <si>
@@ -567,6 +579,9 @@
     <t xml:space="preserve">15:09:47</t>
   </si>
   <si>
+    <t xml:space="preserve">16:22:04</t>
+  </si>
+  <si>
     <t xml:space="preserve">14:27:23</t>
   </si>
   <si>
@@ -616,6 +631,9 @@
   </si>
   <si>
     <t xml:space="preserve">15:08:32</t>
+  </si>
+  <si>
+    <t xml:space="preserve">16:21:34</t>
   </si>
   <si>
     <t xml:space="preserve">11:21:AM</t>
@@ -684,6 +702,9 @@
     <t xml:space="preserve">11:39:59</t>
   </si>
   <si>
+    <t xml:space="preserve">20:51:54</t>
+  </si>
+  <si>
     <t xml:space="preserve">11:17:AM</t>
   </si>
   <si>
@@ -739,6 +760,9 @@
   </si>
   <si>
     <t xml:space="preserve">11:39:55</t>
+  </si>
+  <si>
+    <t xml:space="preserve">20:52:10</t>
   </si>
 </sst>
 </file>
@@ -854,7 +878,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -880,6 +904,10 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1157,7 +1185,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="18" min="18" style="1" width="21.74"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="19" min="19" style="1" width="21.32"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="20" min="20" style="1" width="29.95"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="21" min="21" style="1" width="26.33"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="21" min="21" style="1" width="26.34"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="22" min="22" style="1" width="31.48"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="23" min="23" style="1" width="34.54"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="24" min="24" style="1" width="18.96"/>
@@ -1175,12 +1203,12 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="36" min="36" style="1" width="20.91"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="37" min="37" style="1" width="14.09"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="38" min="38" style="1" width="29.12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="39" min="39" style="1" width="23.14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="39" min="39" style="1" width="23.15"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="40" min="40" style="1" width="16.31"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="41" min="41" style="1" width="31.34"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="42" min="42" style="1" width="21.19"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="43" min="43" style="1" width="13.95"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="44" min="44" style="1" width="29.4"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="44" min="44" style="1" width="29.39"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="45" min="45" style="1" width="22.86"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="46" min="46" style="1" width="15.48"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="47" min="47" style="1" width="31.06"/>
@@ -1203,11 +1231,11 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="64" min="64" style="1" width="12.84"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="65" min="65" style="1" width="31.76"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="66" min="66" style="1" width="20.77"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="67" min="67" style="1" width="10.06"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="67" min="67" style="1" width="10.07"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="68" min="68" style="1" width="28.97"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="69" min="69" style="1" width="21.19"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="70" min="70" style="1" width="10.48"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="71" min="71" style="1" width="29.4"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="70" min="70" style="1" width="10.47"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="71" min="71" style="1" width="29.39"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="72" min="72" style="1" width="22.86"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="73" min="73" style="1" width="12.98"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="74" min="74" style="1" width="31.9"/>
@@ -5500,6 +5528,264 @@
       <c r="CE21" s="1" t="n">
         <v>-59.09</v>
       </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="1" t="n">
+        <v>20</v>
+      </c>
+      <c r="B22" s="1" t="s">
+        <v>143</v>
+      </c>
+      <c r="C22" s="1" t="s">
+        <v>144</v>
+      </c>
+      <c r="D22" s="1" t="s">
+        <v>145</v>
+      </c>
+      <c r="E22" s="1" t="n">
+        <v>100</v>
+      </c>
+      <c r="F22" s="1" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="G22" s="1" t="n">
+        <v>0.19</v>
+      </c>
+      <c r="H22" s="1" t="n">
+        <v>5.56</v>
+      </c>
+      <c r="I22" s="1" t="n">
+        <v>0.48</v>
+      </c>
+      <c r="J22" s="1" t="n">
+        <v>0.24</v>
+      </c>
+      <c r="K22" s="1" t="n">
+        <v>-11.11</v>
+      </c>
+      <c r="L22" s="1" t="n">
+        <v>0.53</v>
+      </c>
+      <c r="M22" s="1" t="n">
+        <v>0.26</v>
+      </c>
+      <c r="N22" s="1" t="n">
+        <v>-3.7</v>
+      </c>
+      <c r="O22" s="1" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="P22" s="1" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="Q22" s="1" t="n">
+        <v>2.56</v>
+      </c>
+      <c r="R22" s="1" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S22" s="1" t="n">
+        <v>0.33</v>
+      </c>
+      <c r="T22" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="U22" s="1" t="n">
+        <v>0.67</v>
+      </c>
+      <c r="V22" s="1" t="n">
+        <v>0.34</v>
+      </c>
+      <c r="W22" s="1" t="n">
+        <v>-8.11</v>
+      </c>
+      <c r="X22" s="1" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="Y22" s="1" t="n">
+        <v>0.21</v>
+      </c>
+      <c r="Z22" s="1" t="n">
+        <v>-12.5</v>
+      </c>
+      <c r="AA22" s="1" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AB22" s="1" t="n">
+        <v>0.29</v>
+      </c>
+      <c r="AC22" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD22" s="1" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="AE22" s="1" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="AF22" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG22" s="1" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AH22" s="1" t="n">
+        <v>0.23</v>
+      </c>
+      <c r="AI22" s="1" t="n">
+        <v>-4.17</v>
+      </c>
+      <c r="AJ22" s="1" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AK22" s="1" t="n">
+        <v>0.19</v>
+      </c>
+      <c r="AL22" s="1" t="n">
+        <v>-5</v>
+      </c>
+      <c r="AM22" s="1" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AN22" s="1" t="n">
+        <v>0.22</v>
+      </c>
+      <c r="AO22" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP22" s="1" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AQ22" s="1" t="n">
+        <v>0.21</v>
+      </c>
+      <c r="AR22" s="1" t="n">
+        <v>-4.55</v>
+      </c>
+      <c r="AS22" s="1" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AT22" s="1" t="n">
+        <v>0.27</v>
+      </c>
+      <c r="AU22" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV22" s="1" t="n">
+        <v>0.78</v>
+      </c>
+      <c r="AW22" s="1" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="AX22" s="1" t="n">
+        <v>-1.69</v>
+      </c>
+      <c r="AY22" s="1" t="n">
+        <v>0.81</v>
+      </c>
+      <c r="AZ22" s="1" t="n">
+        <v>0.19</v>
+      </c>
+      <c r="BA22" s="1" t="n">
+        <v>5.56</v>
+      </c>
+      <c r="BB22" s="1" t="n">
+        <v>0.61</v>
+      </c>
+      <c r="BC22" s="1" t="n">
+        <v>0.18</v>
+      </c>
+      <c r="BD22" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="BE22" s="1" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="BF22" s="1" t="n">
+        <v>0.18</v>
+      </c>
+      <c r="BG22" s="1" t="n">
+        <v>-5.26</v>
+      </c>
+      <c r="BH22" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="BI22" s="5" t="n">
+        <v>2.43</v>
+      </c>
+      <c r="BJ22" s="1" t="n">
+        <v>-2.8</v>
+      </c>
+      <c r="BK22" s="1" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="BL22" s="1" t="n">
+        <v>0.71</v>
+      </c>
+      <c r="BM22" s="1" t="n">
+        <v>1.43</v>
+      </c>
+      <c r="BN22" s="1" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="BO22" s="5" t="n">
+        <v>0.74</v>
+      </c>
+      <c r="BP22" s="1" t="n">
+        <v>12.12</v>
+      </c>
+      <c r="BQ22" s="1" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="BR22" s="1" t="n">
+        <v>0.57</v>
+      </c>
+      <c r="BS22" s="1" t="n">
+        <v>3.64</v>
+      </c>
+      <c r="BT22" s="1" t="n">
+        <v>0.48</v>
+      </c>
+      <c r="BU22" s="1" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="BV22" s="1" t="n">
+        <v>-9.09</v>
+      </c>
+      <c r="BW22" s="1" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="BX22" s="1" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="BY22" s="1" t="n">
+        <v>-10</v>
+      </c>
+      <c r="BZ22" s="1" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="CA22" s="1" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="CB22" s="5" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="CC22" s="1" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="CD22" s="1" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="CE22" s="5" t="n">
+        <v>11.11</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="BI23" s="5"/>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="BI24" s="5"/>
+      <c r="BY24" s="5"/>
     </row>
     <row r="1048547" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="1048548" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
@@ -5551,7 +5837,7 @@
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="13.68"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="10.33"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="10.34"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="11.85"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="10.75"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="15.62"/>
@@ -5569,7 +5855,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="18" min="18" style="1" width="21.74"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="19" min="19" style="1" width="21.32"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="20" min="20" style="1" width="29.95"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="21" min="21" style="1" width="26.33"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="21" min="21" style="1" width="26.34"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="22" min="22" style="1" width="31.48"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="23" min="23" style="1" width="34.54"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="24" min="24" style="1" width="18.96"/>
@@ -5587,12 +5873,12 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="36" min="36" style="1" width="20.91"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="37" min="37" style="1" width="14.09"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="38" min="38" style="1" width="29.12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="39" min="39" style="1" width="23.14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="39" min="39" style="1" width="23.15"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="40" min="40" style="1" width="16.31"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="41" min="41" style="1" width="31.34"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="42" min="42" style="1" width="21.19"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="43" min="43" style="1" width="13.95"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="44" min="44" style="1" width="29.4"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="44" min="44" style="1" width="29.39"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="45" min="45" style="1" width="22.86"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="46" min="46" style="1" width="15.48"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="47" min="47" style="1" width="31.06"/>
@@ -5615,11 +5901,11 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="64" min="64" style="1" width="12.84"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="65" min="65" style="1" width="31.76"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="66" min="66" style="1" width="20.77"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="67" min="67" style="1" width="10.06"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="67" min="67" style="1" width="10.07"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="68" min="68" style="1" width="28.97"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="69" min="69" style="1" width="21.19"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="70" min="70" style="1" width="10.48"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="71" min="71" style="1" width="29.4"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="70" min="70" style="1" width="10.47"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="71" min="71" style="1" width="29.39"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="72" min="72" style="1" width="22.86"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="73" min="73" style="1" width="12.98"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="74" min="74" style="1" width="31.9"/>
@@ -5896,7 +6182,7 @@
         <v>84</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="E2" s="1" t="n">
         <v>15</v>
@@ -5943,7 +6229,7 @@
         <v>87</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
       <c r="E3" s="1" t="n">
         <v>15</v>
@@ -6005,7 +6291,7 @@
         <v>90</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="E4" s="1" t="n">
         <v>15</v>
@@ -6067,7 +6353,7 @@
         <v>93</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="E5" s="1" t="n">
         <v>15</v>
@@ -6207,7 +6493,7 @@
         <v>96</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
       <c r="E6" s="1" t="n">
         <v>15</v>
@@ -6374,7 +6660,7 @@
         <v>102</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
       <c r="E7" s="1" t="n">
         <v>30</v>
@@ -6541,7 +6827,7 @@
         <v>105</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
       <c r="E8" s="1" t="n">
         <v>30</v>
@@ -6708,7 +6994,7 @@
         <v>108</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="E9" s="1" t="n">
         <v>50</v>
@@ -6875,7 +7161,7 @@
         <v>111</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="E10" s="1" t="n">
         <v>100</v>
@@ -7090,7 +7376,7 @@
         <v>114</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="E11" s="1" t="n">
         <v>100</v>
@@ -7305,7 +7591,7 @@
         <v>117</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="E12" s="1" t="n">
         <v>100</v>
@@ -7520,7 +7806,7 @@
         <v>120</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="E13" s="1" t="n">
         <v>100</v>
@@ -7735,7 +8021,7 @@
         <v>123</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="E14" s="1" t="n">
         <v>100</v>
@@ -7950,7 +8236,7 @@
         <v>126</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="E15" s="1" t="n">
         <v>100</v>
@@ -8165,7 +8451,7 @@
         <v>129</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="E16" s="1" t="n">
         <v>100</v>
@@ -8380,7 +8666,7 @@
         <v>132</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="E17" s="1" t="n">
         <v>100</v>
@@ -8595,7 +8881,7 @@
         <v>135</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="E18" s="1" t="n">
         <v>100</v>
@@ -8810,7 +9096,7 @@
         <v>138</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
       <c r="E19" s="1" t="n">
         <v>100</v>
@@ -9025,7 +9311,7 @@
         <v>141</v>
       </c>
       <c r="D20" s="1" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="E20" s="1" t="n">
         <v>100</v>
@@ -9226,6 +9512,221 @@
         <v>0</v>
       </c>
       <c r="CD20" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="1" t="n">
+        <v>19</v>
+      </c>
+      <c r="B21" s="1" t="s">
+        <v>143</v>
+      </c>
+      <c r="C21" s="1" t="s">
+        <v>144</v>
+      </c>
+      <c r="D21" s="1" t="s">
+        <v>165</v>
+      </c>
+      <c r="E21" s="1" t="n">
+        <v>100</v>
+      </c>
+      <c r="F21" s="1" t="n">
+        <v>1.55</v>
+      </c>
+      <c r="G21" s="1" t="n">
+        <v>0.38</v>
+      </c>
+      <c r="H21" s="1" t="n">
+        <v>18.75</v>
+      </c>
+      <c r="I21" s="1" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="J21" s="1" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="K21" s="1" t="n">
+        <v>17.02</v>
+      </c>
+      <c r="L21" s="1" t="n">
+        <v>1.73</v>
+      </c>
+      <c r="M21" s="1" t="n">
+        <v>0.39</v>
+      </c>
+      <c r="N21" s="1" t="n">
+        <v>11.43</v>
+      </c>
+      <c r="O21" s="1" t="n">
+        <v>1.99</v>
+      </c>
+      <c r="P21" s="1" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="Q21" s="5" t="n">
+        <v>100</v>
+      </c>
+      <c r="R21" s="1" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="S21" s="1" t="n">
+        <v>0.38</v>
+      </c>
+      <c r="T21" s="1" t="n">
+        <v>-25.49</v>
+      </c>
+      <c r="U21" s="1" t="n">
+        <v>1.67</v>
+      </c>
+      <c r="V21" s="1" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="W21" s="1" t="n">
+        <v>2.04</v>
+      </c>
+      <c r="X21" s="1" t="n">
+        <v>1.13</v>
+      </c>
+      <c r="Y21" s="1" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="Z21" s="5" t="n">
+        <v>32.35</v>
+      </c>
+      <c r="AA21" s="1" t="n">
+        <v>1.14</v>
+      </c>
+      <c r="AB21" s="1" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="AC21" s="5" t="n">
+        <v>14.29</v>
+      </c>
+      <c r="AD21" s="1" t="n">
+        <v>1.26</v>
+      </c>
+      <c r="AE21" s="1" t="n">
+        <v>0.43</v>
+      </c>
+      <c r="AF21" s="1" t="n">
+        <v>-14</v>
+      </c>
+      <c r="AG21" s="1" t="n">
+        <v>1.14</v>
+      </c>
+      <c r="AH21" s="1" t="n">
+        <v>0.39</v>
+      </c>
+      <c r="AI21" s="1" t="n">
+        <v>5.41</v>
+      </c>
+      <c r="AJ21" s="1" t="n">
+        <v>1.08</v>
+      </c>
+      <c r="AK21" s="1" t="n">
+        <v>0.37</v>
+      </c>
+      <c r="AL21" s="1" t="n">
+        <v>15.62</v>
+      </c>
+      <c r="AM21" s="1" t="n">
+        <v>1.14</v>
+      </c>
+      <c r="AN21" s="1" t="n">
+        <v>0.41</v>
+      </c>
+      <c r="AO21" s="5" t="n">
+        <v>20.59</v>
+      </c>
+      <c r="AP21" s="1" t="n">
+        <v>1.17</v>
+      </c>
+      <c r="AQ21" s="1" t="n">
+        <v>0.36</v>
+      </c>
+      <c r="AR21" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS21" s="1" t="n">
+        <v>1.29</v>
+      </c>
+      <c r="AT21" s="1" t="n">
+        <v>0.39</v>
+      </c>
+      <c r="AU21" s="1" t="n">
+        <v>18.18</v>
+      </c>
+      <c r="AV21" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW21" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY21" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ21" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB21" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC21" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="BE21" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF21" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="BH21" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="BI21" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="BK21" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="BL21" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN21" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="BO21" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="BQ21" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="BR21" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="BT21" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="BU21" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="BW21" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="BX21" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="BZ21" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="CA21" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="CC21" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="CD21" s="1" t="n">
         <v>0</v>
       </c>
     </row>
@@ -9255,7 +9756,7 @@
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="13.68"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="10.33"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="10.34"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="11.85"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="10.75"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="15.62"/>
@@ -9273,7 +9774,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="18" min="18" style="1" width="21.74"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="19" min="19" style="1" width="21.32"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="20" min="20" style="1" width="29.95"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="21" min="21" style="1" width="26.33"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="21" min="21" style="1" width="26.34"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="22" min="22" style="1" width="31.48"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="23" min="23" style="1" width="34.54"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="24" min="24" style="1" width="18.96"/>
@@ -9291,12 +9792,12 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="36" min="36" style="1" width="20.91"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="37" min="37" style="1" width="14.09"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="38" min="38" style="1" width="29.12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="39" min="39" style="1" width="23.14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="39" min="39" style="1" width="23.15"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="40" min="40" style="1" width="16.31"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="41" min="41" style="1" width="31.34"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="42" min="42" style="1" width="21.19"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="43" min="43" style="1" width="13.95"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="44" min="44" style="1" width="29.4"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="44" min="44" style="1" width="29.39"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="45" min="45" style="1" width="22.86"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="46" min="46" style="1" width="15.48"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="47" min="47" style="1" width="31.06"/>
@@ -9319,11 +9820,11 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="64" min="64" style="1" width="12.84"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="65" min="65" style="1" width="31.76"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="66" min="66" style="1" width="20.77"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="67" min="67" style="1" width="10.06"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="67" min="67" style="1" width="10.07"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="68" min="68" style="1" width="28.97"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="69" min="69" style="1" width="21.19"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="70" min="70" style="1" width="10.48"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="71" min="71" style="1" width="29.4"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="70" min="70" style="1" width="10.47"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="71" min="71" style="1" width="29.39"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="72" min="72" style="1" width="22.86"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="73" min="73" style="1" width="12.98"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="74" min="74" style="1" width="31.9"/>
@@ -9600,7 +10101,7 @@
         <v>90</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>162</v>
+        <v>166</v>
       </c>
       <c r="E2" s="1" t="n">
         <v>15</v>
@@ -9647,7 +10148,7 @@
         <v>93</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>163</v>
+        <v>167</v>
       </c>
       <c r="E3" s="1" t="n">
         <v>15</v>
@@ -9787,7 +10288,7 @@
         <v>96</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>164</v>
+        <v>168</v>
       </c>
       <c r="E4" s="1" t="n">
         <v>15</v>
@@ -9966,7 +10467,7 @@
         <v>102</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>165</v>
+        <v>169</v>
       </c>
       <c r="E5" s="1" t="n">
         <v>30</v>
@@ -10145,7 +10646,7 @@
         <v>105</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>166</v>
+        <v>170</v>
       </c>
       <c r="E6" s="1" t="n">
         <v>30</v>
@@ -10324,7 +10825,7 @@
         <v>108</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>167</v>
+        <v>171</v>
       </c>
       <c r="E7" s="1" t="n">
         <v>50</v>
@@ -10503,7 +11004,7 @@
         <v>111</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>168</v>
+        <v>172</v>
       </c>
       <c r="E8" s="1" t="n">
         <v>100</v>
@@ -10706,7 +11207,7 @@
         <v>114</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>169</v>
+        <v>173</v>
       </c>
       <c r="E9" s="1" t="n">
         <v>100</v>
@@ -10949,7 +11450,7 @@
         <v>117</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>170</v>
+        <v>174</v>
       </c>
       <c r="E10" s="1" t="n">
         <v>100</v>
@@ -11200,7 +11701,7 @@
         <v>120</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>171</v>
+        <v>175</v>
       </c>
       <c r="E11" s="1" t="n">
         <v>100</v>
@@ -11451,7 +11952,7 @@
         <v>123</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>172</v>
+        <v>176</v>
       </c>
       <c r="E12" s="1" t="n">
         <v>100</v>
@@ -11702,7 +12203,7 @@
         <v>126</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>173</v>
+        <v>177</v>
       </c>
       <c r="E13" s="1" t="n">
         <v>100</v>
@@ -11953,7 +12454,7 @@
         <v>129</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>174</v>
+        <v>178</v>
       </c>
       <c r="E14" s="1" t="n">
         <v>5</v>
@@ -12204,7 +12705,7 @@
         <v>129</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>175</v>
+        <v>179</v>
       </c>
       <c r="E15" s="1" t="n">
         <v>100</v>
@@ -12455,7 +12956,7 @@
         <v>132</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>176</v>
+        <v>180</v>
       </c>
       <c r="E16" s="1" t="n">
         <v>100</v>
@@ -12706,7 +13207,7 @@
         <v>135</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
       <c r="E17" s="1" t="n">
         <v>100</v>
@@ -12957,7 +13458,7 @@
         <v>138</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>178</v>
+        <v>182</v>
       </c>
       <c r="E18" s="1" t="n">
         <v>100</v>
@@ -13208,7 +13709,7 @@
         <v>141</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>179</v>
+        <v>183</v>
       </c>
       <c r="E19" s="1" t="n">
         <v>100</v>
@@ -13445,6 +13946,257 @@
         <v>0.14</v>
       </c>
       <c r="CE19" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="1" t="n">
+        <v>18</v>
+      </c>
+      <c r="B20" s="1" t="s">
+        <v>143</v>
+      </c>
+      <c r="C20" s="1" t="s">
+        <v>144</v>
+      </c>
+      <c r="D20" s="1" t="s">
+        <v>184</v>
+      </c>
+      <c r="E20" s="1" t="n">
+        <v>100</v>
+      </c>
+      <c r="F20" s="1" t="n">
+        <v>0.33</v>
+      </c>
+      <c r="G20" s="1" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="H20" s="1" t="n">
+        <v>7.14</v>
+      </c>
+      <c r="I20" s="1" t="n">
+        <v>0.52</v>
+      </c>
+      <c r="J20" s="1" t="n">
+        <v>0.17</v>
+      </c>
+      <c r="K20" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="L20" s="1" t="n">
+        <v>0.61</v>
+      </c>
+      <c r="M20" s="1" t="n">
+        <v>0.26</v>
+      </c>
+      <c r="N20" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="O20" s="1" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="P20" s="1" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="Q20" s="1" t="n">
+        <v>-12</v>
+      </c>
+      <c r="R20" s="1" t="n">
+        <v>0.51</v>
+      </c>
+      <c r="S20" s="1" t="n">
+        <v>0.34</v>
+      </c>
+      <c r="T20" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="U20" s="1" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="V20" s="1" t="n">
+        <v>0.21</v>
+      </c>
+      <c r="W20" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="X20" s="1" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="Y20" s="1" t="n">
+        <v>0.17</v>
+      </c>
+      <c r="Z20" s="1" t="n">
+        <v>-5.56</v>
+      </c>
+      <c r="AA20" s="1" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AB20" s="1" t="n">
+        <v>0.23</v>
+      </c>
+      <c r="AC20" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD20" s="1" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AE20" s="1" t="n">
+        <v>0.29</v>
+      </c>
+      <c r="AF20" s="1" t="n">
+        <v>-3.33</v>
+      </c>
+      <c r="AG20" s="1" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AH20" s="1" t="n">
+        <v>0.19</v>
+      </c>
+      <c r="AI20" s="1" t="n">
+        <v>5.56</v>
+      </c>
+      <c r="AJ20" s="1" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AK20" s="1" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="AL20" s="1" t="n">
+        <v>-6.25</v>
+      </c>
+      <c r="AM20" s="1" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AN20" s="1" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="AO20" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP20" s="1" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AQ20" s="1" t="n">
+        <v>0.21</v>
+      </c>
+      <c r="AR20" s="1" t="n">
+        <v>-4.55</v>
+      </c>
+      <c r="AS20" s="1" t="n">
+        <v>0.64</v>
+      </c>
+      <c r="AT20" s="1" t="n">
+        <v>0.27</v>
+      </c>
+      <c r="AU20" s="1" t="n">
+        <v>3.85</v>
+      </c>
+      <c r="AV20" s="1" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="AW20" s="1" t="n">
+        <v>0.67</v>
+      </c>
+      <c r="AX20" s="1" t="n">
+        <v>1.52</v>
+      </c>
+      <c r="AY20" s="1" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="AZ20" s="1" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="BA20" s="1" t="n">
+        <v>-5.41</v>
+      </c>
+      <c r="BB20" s="1" t="n">
+        <v>0.71</v>
+      </c>
+      <c r="BC20" s="1" t="n">
+        <v>0.46</v>
+      </c>
+      <c r="BD20" s="1" t="n">
+        <v>-2.13</v>
+      </c>
+      <c r="BE20" s="1" t="n">
+        <v>0.67</v>
+      </c>
+      <c r="BF20" s="1" t="n">
+        <v>0.31</v>
+      </c>
+      <c r="BG20" s="1" t="n">
+        <v>-3.12</v>
+      </c>
+      <c r="BH20" s="1" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="BI20" s="1" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="BJ20" s="1" t="n">
+        <v>-1.23</v>
+      </c>
+      <c r="BK20" s="1" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="BL20" s="1" t="n">
+        <v>0.27</v>
+      </c>
+      <c r="BM20" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN20" s="1" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="BO20" s="1" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="BP20" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="BQ20" s="1" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="BR20" s="1" t="n">
+        <v>0.36</v>
+      </c>
+      <c r="BS20" s="1" t="n">
+        <v>5.88</v>
+      </c>
+      <c r="BT20" s="1" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="BU20" s="1" t="n">
+        <v>0.27</v>
+      </c>
+      <c r="BV20" s="1" t="n">
+        <v>-6.9</v>
+      </c>
+      <c r="BW20" s="1" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="BX20" s="1" t="n">
+        <v>0.18</v>
+      </c>
+      <c r="BY20" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="BZ20" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="CA20" s="1" t="n">
+        <v>0.18</v>
+      </c>
+      <c r="CB20" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="CC20" s="1" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="CD20" s="1" t="n">
+        <v>0.14</v>
+      </c>
+      <c r="CE20" s="1" t="n">
         <v>0</v>
       </c>
     </row>
@@ -13469,7 +14221,7 @@
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="13.68"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="10.33"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="10.34"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="11.85"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="10.75"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="15.62"/>
@@ -13487,7 +14239,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="18" min="18" style="1" width="21.74"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="19" min="19" style="1" width="21.32"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="20" min="20" style="1" width="29.95"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="21" min="21" style="1" width="26.33"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="21" min="21" style="1" width="26.34"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="22" min="22" style="1" width="31.48"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="23" min="23" style="1" width="34.54"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="24" min="24" style="1" width="18.96"/>
@@ -13505,12 +14257,12 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="36" min="36" style="1" width="20.91"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="37" min="37" style="1" width="14.09"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="38" min="38" style="1" width="29.12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="39" min="39" style="1" width="23.14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="39" min="39" style="1" width="23.15"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="40" min="40" style="1" width="16.31"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="41" min="41" style="1" width="31.34"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="42" min="42" style="1" width="21.19"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="43" min="43" style="1" width="13.95"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="44" min="44" style="1" width="29.4"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="44" min="44" style="1" width="29.39"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="45" min="45" style="1" width="22.86"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="46" min="46" style="1" width="15.48"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="47" min="47" style="1" width="31.06"/>
@@ -13533,11 +14285,11 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="64" min="64" style="1" width="12.84"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="65" min="65" style="1" width="31.76"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="66" min="66" style="1" width="20.77"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="67" min="67" style="1" width="10.06"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="67" min="67" style="1" width="10.07"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="68" min="68" style="1" width="28.97"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="69" min="69" style="1" width="21.19"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="70" min="70" style="1" width="10.48"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="71" min="71" style="1" width="29.4"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="70" min="70" style="1" width="10.47"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="71" min="71" style="1" width="29.39"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="72" min="72" style="1" width="22.86"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="73" min="73" style="1" width="12.98"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="74" min="74" style="1" width="31.9"/>
@@ -13814,7 +14566,7 @@
         <v>90</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>180</v>
+        <v>185</v>
       </c>
       <c r="E2" s="1" t="n">
         <v>15</v>
@@ -13861,7 +14613,7 @@
         <v>93</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>181</v>
+        <v>186</v>
       </c>
       <c r="E3" s="1" t="n">
         <v>15</v>
@@ -14001,7 +14753,7 @@
         <v>96</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>182</v>
+        <v>187</v>
       </c>
       <c r="E4" s="1" t="n">
         <v>15</v>
@@ -14168,7 +14920,7 @@
         <v>102</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>183</v>
+        <v>188</v>
       </c>
       <c r="E5" s="1" t="n">
         <v>30</v>
@@ -14335,7 +15087,7 @@
         <v>105</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>184</v>
+        <v>189</v>
       </c>
       <c r="E6" s="1" t="n">
         <v>30</v>
@@ -14502,7 +15254,7 @@
         <v>108</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>185</v>
+        <v>190</v>
       </c>
       <c r="E7" s="1" t="n">
         <v>50</v>
@@ -14669,7 +15421,7 @@
         <v>111</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>186</v>
+        <v>191</v>
       </c>
       <c r="E8" s="1" t="n">
         <v>100</v>
@@ -14884,7 +15636,7 @@
         <v>114</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>187</v>
+        <v>192</v>
       </c>
       <c r="E9" s="1" t="n">
         <v>100</v>
@@ -15099,7 +15851,7 @@
         <v>117</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>188</v>
+        <v>193</v>
       </c>
       <c r="E10" s="1" t="n">
         <v>100</v>
@@ -15314,7 +16066,7 @@
         <v>120</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>189</v>
+        <v>194</v>
       </c>
       <c r="E11" s="1" t="n">
         <v>100</v>
@@ -15529,7 +16281,7 @@
         <v>123</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>190</v>
+        <v>195</v>
       </c>
       <c r="E12" s="1" t="n">
         <v>100</v>
@@ -15744,7 +16496,7 @@
         <v>126</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>191</v>
+        <v>196</v>
       </c>
       <c r="E13" s="1" t="n">
         <v>100</v>
@@ -15959,7 +16711,7 @@
         <v>129</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>192</v>
+        <v>197</v>
       </c>
       <c r="E14" s="1" t="n">
         <v>100</v>
@@ -16174,7 +16926,7 @@
         <v>132</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>193</v>
+        <v>198</v>
       </c>
       <c r="E15" s="1" t="n">
         <v>100</v>
@@ -16389,7 +17141,7 @@
         <v>135</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>194</v>
+        <v>199</v>
       </c>
       <c r="E16" s="1" t="n">
         <v>100</v>
@@ -16604,7 +17356,7 @@
         <v>138</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>195</v>
+        <v>200</v>
       </c>
       <c r="E17" s="1" t="n">
         <v>100</v>
@@ -16819,7 +17571,7 @@
         <v>141</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>196</v>
+        <v>201</v>
       </c>
       <c r="E18" s="1" t="n">
         <v>100</v>
@@ -17020,6 +17772,221 @@
         <v>0</v>
       </c>
       <c r="CD18" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="1" t="n">
+        <v>17</v>
+      </c>
+      <c r="B19" s="1" t="s">
+        <v>143</v>
+      </c>
+      <c r="C19" s="1" t="s">
+        <v>144</v>
+      </c>
+      <c r="D19" s="1" t="s">
+        <v>202</v>
+      </c>
+      <c r="E19" s="1" t="n">
+        <v>100</v>
+      </c>
+      <c r="F19" s="1" t="n">
+        <v>1.49</v>
+      </c>
+      <c r="G19" s="1" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="H19" s="1" t="n">
+        <v>2.94</v>
+      </c>
+      <c r="I19" s="1" t="n">
+        <v>1.81</v>
+      </c>
+      <c r="J19" s="1" t="n">
+        <v>0.43</v>
+      </c>
+      <c r="K19" s="1" t="n">
+        <v>-6.52</v>
+      </c>
+      <c r="L19" s="1" t="n">
+        <v>1.77</v>
+      </c>
+      <c r="M19" s="1" t="n">
+        <v>0.39</v>
+      </c>
+      <c r="N19" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="O19" s="1" t="n">
+        <v>2.05</v>
+      </c>
+      <c r="P19" s="1" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="Q19" s="7" t="n">
+        <v>32.35</v>
+      </c>
+      <c r="R19" s="1" t="n">
+        <v>1.89</v>
+      </c>
+      <c r="S19" s="1" t="n">
+        <v>0.48</v>
+      </c>
+      <c r="T19" s="1" t="n">
+        <v>-12.73</v>
+      </c>
+      <c r="U19" s="1" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="V19" s="1" t="n">
+        <v>0.48</v>
+      </c>
+      <c r="W19" s="1" t="n">
+        <v>17.07</v>
+      </c>
+      <c r="X19" s="1" t="n">
+        <v>1.55</v>
+      </c>
+      <c r="Y19" s="1" t="n">
+        <v>0.33</v>
+      </c>
+      <c r="Z19" s="1" t="n">
+        <v>-19.51</v>
+      </c>
+      <c r="AA19" s="1" t="n">
+        <v>1.43</v>
+      </c>
+      <c r="AB19" s="1" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="AC19" s="1" t="n">
+        <v>6.06</v>
+      </c>
+      <c r="AD19" s="1" t="n">
+        <v>1.62</v>
+      </c>
+      <c r="AE19" s="1" t="n">
+        <v>0.42</v>
+      </c>
+      <c r="AF19" s="1" t="n">
+        <v>-6.67</v>
+      </c>
+      <c r="AG19" s="1" t="n">
+        <v>1.62</v>
+      </c>
+      <c r="AH19" s="1" t="n">
+        <v>0.39</v>
+      </c>
+      <c r="AI19" s="1" t="n">
+        <v>2.63</v>
+      </c>
+      <c r="AJ19" s="1" t="n">
+        <v>1.68</v>
+      </c>
+      <c r="AK19" s="1" t="n">
+        <v>0.33</v>
+      </c>
+      <c r="AL19" s="1" t="n">
+        <v>3.12</v>
+      </c>
+      <c r="AM19" s="1" t="n">
+        <v>1.46</v>
+      </c>
+      <c r="AN19" s="1" t="n">
+        <v>0.37</v>
+      </c>
+      <c r="AO19" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP19" s="1" t="n">
+        <v>1.37</v>
+      </c>
+      <c r="AQ19" s="1" t="n">
+        <v>0.41</v>
+      </c>
+      <c r="AR19" s="1" t="n">
+        <v>-14.58</v>
+      </c>
+      <c r="AS19" s="1" t="n">
+        <v>1.78</v>
+      </c>
+      <c r="AT19" s="1" t="n">
+        <v>0.38</v>
+      </c>
+      <c r="AU19" s="1" t="n">
+        <v>-5</v>
+      </c>
+      <c r="AV19" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW19" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY19" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ19" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB19" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC19" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="BE19" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF19" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="BH19" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="BI19" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="BK19" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="BL19" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN19" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="BO19" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="BQ19" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="BR19" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="BT19" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="BU19" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="BW19" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="BX19" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="BZ19" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="CA19" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="CC19" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="CD19" s="1" t="n">
         <v>0</v>
       </c>
     </row>
@@ -17062,7 +18029,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="18" min="18" style="1" width="21.74"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="19" min="19" style="1" width="21.32"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="20" min="20" style="1" width="29.95"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="21" min="21" style="1" width="26.33"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="21" min="21" style="1" width="26.34"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="22" min="22" style="1" width="31.48"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="23" min="23" style="1" width="34.54"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="24" min="24" style="1" width="18.96"/>
@@ -17080,12 +18047,12 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="36" min="36" style="1" width="20.91"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="37" min="37" style="1" width="14.09"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="38" min="38" style="1" width="29.12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="39" min="39" style="1" width="23.14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="39" min="39" style="1" width="23.15"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="40" min="40" style="1" width="16.31"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="41" min="41" style="1" width="31.34"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="42" min="42" style="1" width="21.19"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="43" min="43" style="1" width="13.95"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="44" min="44" style="1" width="29.4"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="44" min="44" style="1" width="29.39"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="45" min="45" style="1" width="22.86"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="46" min="46" style="1" width="15.48"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="47" min="47" style="1" width="31.06"/>
@@ -17108,11 +18075,11 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="64" min="64" style="1" width="12.84"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="65" min="65" style="1" width="31.76"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="66" min="66" style="1" width="20.77"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="67" min="67" style="1" width="10.06"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="67" min="67" style="1" width="10.07"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="68" min="68" style="1" width="28.97"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="69" min="69" style="1" width="21.19"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="70" min="70" style="1" width="10.48"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="71" min="71" style="1" width="29.4"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="70" min="70" style="1" width="10.47"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="71" min="71" style="1" width="29.39"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="72" min="72" style="1" width="22.86"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="73" min="73" style="1" width="12.98"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="74" min="74" style="1" width="31.9"/>
@@ -17389,7 +18356,7 @@
         <v>84</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>197</v>
+        <v>203</v>
       </c>
       <c r="E2" s="1" t="n">
         <v>15</v>
@@ -17436,7 +18403,7 @@
         <v>87</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>198</v>
+        <v>204</v>
       </c>
       <c r="E3" s="1" t="n">
         <v>15</v>
@@ -17498,7 +18465,7 @@
         <v>90</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>199</v>
+        <v>205</v>
       </c>
       <c r="E4" s="1" t="n">
         <v>15</v>
@@ -17560,7 +18527,7 @@
         <v>93</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>200</v>
+        <v>206</v>
       </c>
       <c r="E5" s="1" t="n">
         <v>15</v>
@@ -17700,7 +18667,7 @@
         <v>96</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>201</v>
+        <v>207</v>
       </c>
       <c r="E6" s="1" t="n">
         <v>15</v>
@@ -17879,7 +18846,7 @@
         <v>102</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>202</v>
+        <v>208</v>
       </c>
       <c r="E7" s="1" t="n">
         <v>30</v>
@@ -18058,7 +19025,7 @@
         <v>105</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>203</v>
+        <v>209</v>
       </c>
       <c r="E8" s="1" t="n">
         <v>30</v>
@@ -18237,7 +19204,7 @@
         <v>108</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>204</v>
+        <v>210</v>
       </c>
       <c r="E9" s="1" t="n">
         <v>50</v>
@@ -18416,7 +19383,7 @@
         <v>111</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>205</v>
+        <v>211</v>
       </c>
       <c r="E10" s="1" t="n">
         <v>100</v>
@@ -18625,7 +19592,7 @@
         <v>114</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>206</v>
+        <v>212</v>
       </c>
       <c r="E11" s="1" t="n">
         <v>100</v>
@@ -18835,7 +19802,7 @@
         <v>0.29</v>
       </c>
       <c r="BV11" s="5" t="s">
-        <v>207</v>
+        <v>213</v>
       </c>
       <c r="BW11" s="1" t="n">
         <v>0.8</v>
@@ -18867,10 +19834,10 @@
         <v>116</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>208</v>
+        <v>214</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>209</v>
+        <v>215</v>
       </c>
       <c r="E12" s="1" t="n">
         <v>100</v>
@@ -19121,7 +20088,7 @@
         <v>120</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>210</v>
+        <v>216</v>
       </c>
       <c r="E13" s="1" t="n">
         <v>100</v>
@@ -19372,7 +20339,7 @@
         <v>123</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>211</v>
+        <v>217</v>
       </c>
       <c r="E14" s="1" t="n">
         <v>100</v>
@@ -19623,7 +20590,7 @@
         <v>126</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>212</v>
+        <v>218</v>
       </c>
       <c r="E15" s="1" t="n">
         <v>100</v>
@@ -19874,7 +20841,7 @@
         <v>129</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>213</v>
+        <v>219</v>
       </c>
       <c r="E16" s="1" t="n">
         <v>100</v>
@@ -20125,7 +21092,7 @@
         <v>132</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>214</v>
+        <v>220</v>
       </c>
       <c r="E17" s="1" t="n">
         <v>100</v>
@@ -20376,7 +21343,7 @@
         <v>135</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>215</v>
+        <v>221</v>
       </c>
       <c r="E18" s="1" t="n">
         <v>100</v>
@@ -20627,7 +21594,7 @@
         <v>138</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>216</v>
+        <v>222</v>
       </c>
       <c r="E19" s="1" t="n">
         <v>100</v>
@@ -20867,7 +21834,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="1" t="n">
         <v>18</v>
       </c>
@@ -20875,10 +21842,10 @@
         <v>140</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>217</v>
+        <v>223</v>
       </c>
       <c r="D20" s="1" t="s">
-        <v>218</v>
+        <v>224</v>
       </c>
       <c r="E20" s="1" t="n">
         <v>100</v>
@@ -21116,6 +22083,257 @@
       </c>
       <c r="CE20" s="1" t="n">
         <v>-6.67</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="1" t="n">
+        <v>19</v>
+      </c>
+      <c r="B21" s="1" t="s">
+        <v>143</v>
+      </c>
+      <c r="C21" s="1" t="s">
+        <v>144</v>
+      </c>
+      <c r="D21" s="1" t="s">
+        <v>225</v>
+      </c>
+      <c r="E21" s="1" t="n">
+        <v>100</v>
+      </c>
+      <c r="F21" s="1" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="G21" s="1" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="H21" s="1" t="n">
+        <v>15.38</v>
+      </c>
+      <c r="I21" s="1" t="n">
+        <v>0.51</v>
+      </c>
+      <c r="J21" s="1" t="n">
+        <v>0.18</v>
+      </c>
+      <c r="K21" s="1" t="n">
+        <v>5.88</v>
+      </c>
+      <c r="L21" s="1" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="M21" s="1" t="n">
+        <v>0.27</v>
+      </c>
+      <c r="N21" s="1" t="n">
+        <v>3.85</v>
+      </c>
+      <c r="O21" s="1" t="n">
+        <v>0.68</v>
+      </c>
+      <c r="P21" s="1" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="Q21" s="1" t="n">
+        <v>2.08</v>
+      </c>
+      <c r="R21" s="1" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="S21" s="1" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="T21" s="1" t="n">
+        <v>-2.78</v>
+      </c>
+      <c r="U21" s="1" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="V21" s="1" t="n">
+        <v>0.22</v>
+      </c>
+      <c r="W21" s="1" t="n">
+        <v>15.79</v>
+      </c>
+      <c r="X21" s="1" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="Y21" s="1" t="n">
+        <v>0.19</v>
+      </c>
+      <c r="Z21" s="1" t="n">
+        <v>5.56</v>
+      </c>
+      <c r="AA21" s="1" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AB21" s="1" t="n">
+        <v>0.24</v>
+      </c>
+      <c r="AC21" s="1" t="n">
+        <v>-4</v>
+      </c>
+      <c r="AD21" s="1" t="n">
+        <v>0.64</v>
+      </c>
+      <c r="AE21" s="1" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="AF21" s="1" t="n">
+        <v>3.45</v>
+      </c>
+      <c r="AG21" s="1" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AH21" s="1" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="AI21" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ21" s="1" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AK21" s="1" t="n">
+        <v>0.17</v>
+      </c>
+      <c r="AL21" s="1" t="n">
+        <v>6.25</v>
+      </c>
+      <c r="AM21" s="1" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AN21" s="1" t="n">
+        <v>0.26</v>
+      </c>
+      <c r="AO21" s="1" t="n">
+        <v>13.04</v>
+      </c>
+      <c r="AP21" s="1" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AQ21" s="1" t="n">
+        <v>0.21</v>
+      </c>
+      <c r="AR21" s="1" t="n">
+        <v>-4.55</v>
+      </c>
+      <c r="AS21" s="1" t="n">
+        <v>0.59</v>
+      </c>
+      <c r="AT21" s="1" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="AU21" s="1" t="n">
+        <v>3.7</v>
+      </c>
+      <c r="AV21" s="1" t="n">
+        <v>0.86</v>
+      </c>
+      <c r="AW21" s="1" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="AX21" s="1" t="n">
+        <v>-2.94</v>
+      </c>
+      <c r="AY21" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="AZ21" s="1" t="n">
+        <v>0.69</v>
+      </c>
+      <c r="BA21" s="1" t="n">
+        <v>-2.82</v>
+      </c>
+      <c r="BB21" s="1" t="n">
+        <v>0.69</v>
+      </c>
+      <c r="BC21" s="1" t="n">
+        <v>0.47</v>
+      </c>
+      <c r="BD21" s="1" t="n">
+        <v>-4.08</v>
+      </c>
+      <c r="BE21" s="1" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="BF21" s="1" t="n">
+        <v>0.32</v>
+      </c>
+      <c r="BG21" s="1" t="n">
+        <v>-3.03</v>
+      </c>
+      <c r="BH21" s="1" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="BI21" s="1" t="n">
+        <v>0.81</v>
+      </c>
+      <c r="BJ21" s="1" t="n">
+        <v>-1.22</v>
+      </c>
+      <c r="BK21" s="1" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="BL21" s="1" t="n">
+        <v>0.27</v>
+      </c>
+      <c r="BM21" s="1" t="n">
+        <v>-6.9</v>
+      </c>
+      <c r="BN21" s="1" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="BO21" s="1" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="BP21" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="BQ21" s="1" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="BR21" s="1" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="BS21" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="BT21" s="1" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="BU21" s="1" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="BV21" s="1" t="n">
+        <v>7.69</v>
+      </c>
+      <c r="BW21" s="1" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="BX21" s="1" t="n">
+        <v>0.19</v>
+      </c>
+      <c r="BY21" s="1" t="n">
+        <v>5.56</v>
+      </c>
+      <c r="BZ21" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="CA21" s="1" t="n">
+        <v>0.18</v>
+      </c>
+      <c r="CB21" s="1" t="n">
+        <v>5.88</v>
+      </c>
+      <c r="CC21" s="1" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="CD21" s="1" t="n">
+        <v>0.14</v>
+      </c>
+      <c r="CE21" s="1" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="1048569" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
@@ -21146,7 +22364,7 @@
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="13.68"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="10.33"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="10.34"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="11.85"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="10.75"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="15.62"/>
@@ -21164,7 +22382,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="18" min="18" style="1" width="21.74"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="19" min="19" style="1" width="21.32"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="20" min="20" style="1" width="29.95"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="21" min="21" style="1" width="26.33"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="21" min="21" style="1" width="26.34"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="22" min="22" style="1" width="31.48"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="23" min="23" style="1" width="34.54"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="24" min="24" style="1" width="18.96"/>
@@ -21182,12 +22400,12 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="36" min="36" style="1" width="20.91"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="37" min="37" style="1" width="14.09"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="38" min="38" style="1" width="29.12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="39" min="39" style="1" width="23.14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="39" min="39" style="1" width="23.15"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="40" min="40" style="1" width="16.31"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="41" min="41" style="1" width="31.34"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="42" min="42" style="1" width="21.19"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="43" min="43" style="1" width="13.95"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="44" min="44" style="1" width="29.4"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="44" min="44" style="1" width="29.39"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="45" min="45" style="1" width="22.86"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="46" min="46" style="1" width="15.48"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="47" min="47" style="1" width="31.06"/>
@@ -21210,11 +22428,11 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="64" min="64" style="1" width="12.84"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="65" min="65" style="1" width="31.76"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="66" min="66" style="1" width="20.77"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="67" min="67" style="1" width="10.06"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="67" min="67" style="1" width="10.07"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="68" min="68" style="1" width="28.97"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="69" min="69" style="1" width="21.19"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="70" min="70" style="1" width="10.48"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="71" min="71" style="1" width="29.4"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="70" min="70" style="1" width="10.47"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="71" min="71" style="1" width="29.39"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="72" min="72" style="1" width="22.86"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="73" min="73" style="1" width="12.98"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="74" min="74" style="1" width="31.9"/>
@@ -21491,7 +22709,7 @@
         <v>84</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>219</v>
+        <v>226</v>
       </c>
       <c r="E2" s="1" t="n">
         <v>15</v>
@@ -21538,7 +22756,7 @@
         <v>87</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>220</v>
+        <v>227</v>
       </c>
       <c r="E3" s="1" t="n">
         <v>15</v>
@@ -21600,7 +22818,7 @@
         <v>90</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>221</v>
+        <v>228</v>
       </c>
       <c r="E4" s="1" t="n">
         <v>15</v>
@@ -21662,7 +22880,7 @@
         <v>93</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>222</v>
+        <v>229</v>
       </c>
       <c r="E5" s="1" t="n">
         <v>15</v>
@@ -21802,7 +23020,7 @@
         <v>96</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>223</v>
+        <v>230</v>
       </c>
       <c r="E6" s="1" t="n">
         <v>15</v>
@@ -21969,7 +23187,7 @@
         <v>102</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>224</v>
+        <v>231</v>
       </c>
       <c r="E7" s="1" t="n">
         <v>30</v>
@@ -22136,7 +23354,7 @@
         <v>105</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>225</v>
+        <v>232</v>
       </c>
       <c r="E8" s="1" t="n">
         <v>30</v>
@@ -22303,7 +23521,7 @@
         <v>108</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>226</v>
+        <v>233</v>
       </c>
       <c r="E9" s="1" t="n">
         <v>50</v>
@@ -22470,7 +23688,7 @@
         <v>111</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>227</v>
+        <v>234</v>
       </c>
       <c r="E10" s="1" t="n">
         <v>100</v>
@@ -22685,7 +23903,7 @@
         <v>114</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>228</v>
+        <v>235</v>
       </c>
       <c r="E11" s="1" t="n">
         <v>100</v>
@@ -22897,10 +24115,10 @@
         <v>116</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>208</v>
+        <v>214</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>229</v>
+        <v>236</v>
       </c>
       <c r="E12" s="1" t="n">
         <v>100</v>
@@ -23115,7 +24333,7 @@
         <v>120</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>230</v>
+        <v>237</v>
       </c>
       <c r="E13" s="1" t="n">
         <v>100</v>
@@ -23330,7 +24548,7 @@
         <v>123</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>231</v>
+        <v>238</v>
       </c>
       <c r="E14" s="1" t="n">
         <v>100</v>
@@ -23545,7 +24763,7 @@
         <v>126</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>232</v>
+        <v>239</v>
       </c>
       <c r="E15" s="1" t="n">
         <v>100</v>
@@ -23760,7 +24978,7 @@
         <v>129</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>233</v>
+        <v>240</v>
       </c>
       <c r="E16" s="1" t="n">
         <v>100</v>
@@ -23975,7 +25193,7 @@
         <v>132</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>234</v>
+        <v>241</v>
       </c>
       <c r="E17" s="1" t="n">
         <v>100</v>
@@ -24190,7 +25408,7 @@
         <v>135</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>235</v>
+        <v>242</v>
       </c>
       <c r="E18" s="1" t="n">
         <v>100</v>
@@ -24405,7 +25623,7 @@
         <v>138</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>236</v>
+        <v>243</v>
       </c>
       <c r="E19" s="1" t="n">
         <v>100</v>
@@ -24609,7 +25827,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="1" t="n">
         <v>18</v>
       </c>
@@ -24617,10 +25835,10 @@
         <v>140</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>217</v>
+        <v>223</v>
       </c>
       <c r="D20" s="1" t="s">
-        <v>237</v>
+        <v>244</v>
       </c>
       <c r="E20" s="1" t="n">
         <v>100</v>
@@ -24821,6 +26039,221 @@
         <v>0</v>
       </c>
       <c r="CD20" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="1" t="n">
+        <v>19</v>
+      </c>
+      <c r="B21" s="1" t="s">
+        <v>143</v>
+      </c>
+      <c r="C21" s="1" t="s">
+        <v>144</v>
+      </c>
+      <c r="D21" s="1" t="s">
+        <v>245</v>
+      </c>
+      <c r="E21" s="1" t="n">
+        <v>100</v>
+      </c>
+      <c r="F21" s="1" t="n">
+        <v>1.64</v>
+      </c>
+      <c r="G21" s="1" t="n">
+        <v>0.34</v>
+      </c>
+      <c r="H21" s="1" t="n">
+        <v>-2.86</v>
+      </c>
+      <c r="I21" s="1" t="n">
+        <v>1.63</v>
+      </c>
+      <c r="J21" s="1" t="n">
+        <v>0.37</v>
+      </c>
+      <c r="K21" s="1" t="n">
+        <v>-11.9</v>
+      </c>
+      <c r="L21" s="1" t="n">
+        <v>1.79</v>
+      </c>
+      <c r="M21" s="1" t="n">
+        <v>0.39</v>
+      </c>
+      <c r="N21" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="O21" s="1" t="n">
+        <v>2.41</v>
+      </c>
+      <c r="P21" s="1" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="Q21" s="1" t="n">
+        <v>-10.26</v>
+      </c>
+      <c r="R21" s="1" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="S21" s="1" t="n">
+        <v>0.57</v>
+      </c>
+      <c r="T21" s="1" t="n">
+        <v>18.75</v>
+      </c>
+      <c r="U21" s="1" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="V21" s="1" t="n">
+        <v>0.42</v>
+      </c>
+      <c r="W21" s="1" t="n">
+        <v>-12.5</v>
+      </c>
+      <c r="X21" s="1" t="n">
+        <v>1.43</v>
+      </c>
+      <c r="Y21" s="1" t="n">
+        <v>0.33</v>
+      </c>
+      <c r="Z21" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA21" s="1" t="n">
+        <v>1.47</v>
+      </c>
+      <c r="AB21" s="1" t="n">
+        <v>0.32</v>
+      </c>
+      <c r="AC21" s="1" t="n">
+        <v>-3.03</v>
+      </c>
+      <c r="AD21" s="1" t="n">
+        <v>1.67</v>
+      </c>
+      <c r="AE21" s="1" t="n">
+        <v>0.43</v>
+      </c>
+      <c r="AF21" s="1" t="n">
+        <v>-6.52</v>
+      </c>
+      <c r="AG21" s="1" t="n">
+        <v>1.45</v>
+      </c>
+      <c r="AH21" s="1" t="n">
+        <v>0.37</v>
+      </c>
+      <c r="AI21" s="1" t="n">
+        <v>-2.63</v>
+      </c>
+      <c r="AJ21" s="1" t="n">
+        <v>1.37</v>
+      </c>
+      <c r="AK21" s="1" t="n">
+        <v>0.32</v>
+      </c>
+      <c r="AL21" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM21" s="1" t="n">
+        <v>1.31</v>
+      </c>
+      <c r="AN21" s="1" t="n">
+        <v>0.36</v>
+      </c>
+      <c r="AO21" s="1" t="n">
+        <v>-7.69</v>
+      </c>
+      <c r="AP21" s="1" t="n">
+        <v>1.33</v>
+      </c>
+      <c r="AQ21" s="1" t="n">
+        <v>0.39</v>
+      </c>
+      <c r="AR21" s="1" t="n">
+        <v>-9.3</v>
+      </c>
+      <c r="AS21" s="1" t="n">
+        <v>1.75</v>
+      </c>
+      <c r="AT21" s="1" t="n">
+        <v>0.39</v>
+      </c>
+      <c r="AU21" s="1" t="n">
+        <v>-4.88</v>
+      </c>
+      <c r="AV21" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW21" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY21" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ21" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB21" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC21" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="BE21" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF21" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="BH21" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="BI21" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="BK21" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="BL21" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN21" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="BO21" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="BQ21" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="BR21" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="BT21" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="BU21" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="BW21" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="BX21" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="BZ21" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="CA21" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="CC21" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="CD21" s="1" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>